<commit_message>
Change buck to have 20uF Cout, increase inductor footprint size
</commit_message>
<xml_diff>
--- a/eagle/bom/bom_jlc.xlsx
+++ b/eagle/bom/bom_jlc.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wpi0-my.sharepoint.com/personal/jwbuchta_wpi_edu/Documents/Jobs/academic_technician/flashing_led/eagle/bom/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="39" documentId="11_F25DC773A252ABDACC10483079DB61465BDE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{67624739-4B7A-4EC9-ABB4-87E15845DA2A}"/>
+  <xr:revisionPtr revIDLastSave="40" documentId="11_F25DC773A252ABDACC10483079DB61465BDE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{23C8A960-41FB-4581-B704-65B1E1C7A0EE}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="66">
   <si>
     <t>Qty</t>
   </si>
@@ -162,9 +162,6 @@
   </si>
   <si>
     <t>TPS63002DRCR</t>
-  </si>
-  <si>
-    <t>TPS63001DRCR</t>
   </si>
   <si>
     <t>VREG_V62/16624-01YE</t>
@@ -632,7 +629,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -644,7 +641,7 @@
         <v>3</v>
       </c>
       <c r="F1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -664,7 +661,7 @@
         <v>7</v>
       </c>
       <c r="F2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="72" x14ac:dyDescent="0.55000000000000004">
@@ -681,10 +678,10 @@
         <v>9</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -704,7 +701,7 @@
         <v>11</v>
       </c>
       <c r="F4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -724,7 +721,7 @@
         <v>15</v>
       </c>
       <c r="F5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -744,7 +741,7 @@
         <v>19</v>
       </c>
       <c r="F6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -764,7 +761,7 @@
         <v>21</v>
       </c>
       <c r="F7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -784,7 +781,7 @@
         <v>24</v>
       </c>
       <c r="F8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -804,7 +801,7 @@
         <v>26</v>
       </c>
       <c r="F9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -824,7 +821,7 @@
         <v>29</v>
       </c>
       <c r="F10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -844,7 +841,7 @@
         <v>32</v>
       </c>
       <c r="F11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -864,7 +861,7 @@
         <v>35</v>
       </c>
       <c r="F12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="86.4" x14ac:dyDescent="0.55000000000000004">
@@ -881,10 +878,10 @@
         <v>37</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F13" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -904,7 +901,7 @@
         <v>40</v>
       </c>
       <c r="F14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -915,16 +912,16 @@
         <v>41</v>
       </c>
       <c r="C15" t="s">
+        <v>41</v>
+      </c>
+      <c r="D15" t="s">
         <v>42</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>43</v>
       </c>
-      <c r="E15" t="s">
-        <v>44</v>
-      </c>
       <c r="F15" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -932,19 +929,19 @@
         <v>1</v>
       </c>
       <c r="B16" t="s">
+        <v>44</v>
+      </c>
+      <c r="C16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" t="s">
         <v>45</v>
       </c>
-      <c r="C16" t="s">
-        <v>45</v>
-      </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>46</v>
       </c>
-      <c r="E16" t="s">
-        <v>47</v>
-      </c>
       <c r="F16" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add resistive feedback to TP63000
</commit_message>
<xml_diff>
--- a/eagle/bom/bom_jlc.xlsx
+++ b/eagle/bom/bom_jlc.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wpi0-my.sharepoint.com/personal/jwbuchta_wpi_edu/Documents/Jobs/academic_technician/flashing_led/eagle/bom/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="40" documentId="11_F25DC773A252ABDACC10483079DB61465BDE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{23C8A960-41FB-4581-B704-65B1E1C7A0EE}"/>
+  <xr:revisionPtr revIDLastSave="54" documentId="11_F25DC773A252ABDACC10483079DB61465BDE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{79D2FDBF-B5C6-4A75-A15A-79B1FA6E96C4}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="-7500" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="reva" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="ExternalData_1" localSheetId="0" hidden="1">'reva'!$A$1:$F$16</definedName>
+    <definedName name="ExternalData_1" localSheetId="0" hidden="1">'reva'!$A$1:$F$17</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="69">
   <si>
     <t>Qty</t>
   </si>
@@ -116,9 +116,6 @@
     <t>75k</t>
   </si>
   <si>
-    <t>R96, R97, R109</t>
-  </si>
-  <si>
     <t>CR2450</t>
   </si>
   <si>
@@ -159,9 +156,6 @@
   </si>
   <si>
     <t>PWR</t>
-  </si>
-  <si>
-    <t>TPS63002DRCR</t>
   </si>
   <si>
     <t>VREG_V62/16624-01YE</t>
@@ -209,9 +203,6 @@
     <t xml:space="preserve">Value </t>
   </si>
   <si>
-    <t>C116655</t>
-  </si>
-  <si>
     <t>C165948</t>
   </si>
   <si>
@@ -243,6 +234,24 @@
   </si>
   <si>
     <t>C25117</t>
+  </si>
+  <si>
+    <t>C24966</t>
+  </si>
+  <si>
+    <t>TPS63000DRCR</t>
+  </si>
+  <si>
+    <t>680k</t>
+  </si>
+  <si>
+    <t>C4131</t>
+  </si>
+  <si>
+    <t>R76</t>
+  </si>
+  <si>
+    <t>R96, R97, R109, R110</t>
   </si>
 </sst>
 </file>
@@ -336,8 +345,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{90424B35-5CEB-4CD6-81EE-F5B24B27F562}" name="reva" displayName="reva" ref="A1:F16" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:F16" xr:uid="{90424B35-5CEB-4CD6-81EE-F5B24B27F562}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{90424B35-5CEB-4CD6-81EE-F5B24B27F562}" name="reva" displayName="reva" ref="A1:F17" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:F17" xr:uid="{90424B35-5CEB-4CD6-81EE-F5B24B27F562}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{2476360E-FF06-4F0C-9637-377C5ECEE43B}" uniqueName="1" name="Qty" queryTableFieldId="1"/>
     <tableColumn id="2" xr3:uid="{2767049D-B033-4344-BDD3-0987A48978DC}" uniqueName="2" name="Value " queryTableFieldId="2" dataDxfId="4"/>
@@ -613,7 +622,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{037C7287-9E61-4DDA-934D-4945F03370EA}">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="5.83984375" bestFit="1" customWidth="1"/>
@@ -629,7 +638,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -641,7 +650,7 @@
         <v>3</v>
       </c>
       <c r="F1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -661,7 +670,7 @@
         <v>7</v>
       </c>
       <c r="F2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="72" x14ac:dyDescent="0.55000000000000004">
@@ -678,10 +687,10 @@
         <v>9</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F3" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -701,7 +710,7 @@
         <v>11</v>
       </c>
       <c r="F4" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -721,7 +730,7 @@
         <v>15</v>
       </c>
       <c r="F5" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -741,7 +750,7 @@
         <v>19</v>
       </c>
       <c r="F6" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -761,7 +770,7 @@
         <v>21</v>
       </c>
       <c r="F7" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -781,15 +790,15 @@
         <v>24</v>
       </c>
       <c r="F8" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A9">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
+        <v>65</v>
       </c>
       <c r="C9" t="s">
         <v>8</v>
@@ -798,30 +807,30 @@
         <v>9</v>
       </c>
       <c r="E9" t="s">
-        <v>26</v>
+        <v>67</v>
       </c>
       <c r="F9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A10">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B10" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C10" t="s">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="D10" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="E10" t="s">
-        <v>29</v>
+        <v>68</v>
       </c>
       <c r="F10" t="s">
-        <v>50</v>
+        <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -829,19 +838,19 @@
         <v>1</v>
       </c>
       <c r="B11" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C11" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="D11" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="E11" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="F11" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -849,59 +858,59 @@
         <v>1</v>
       </c>
       <c r="B12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" t="s">
+        <v>29</v>
+      </c>
+      <c r="D12" t="s">
+        <v>30</v>
+      </c>
+      <c r="E12" t="s">
+        <v>31</v>
+      </c>
+      <c r="F12" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A13">
+        <v>1</v>
+      </c>
+      <c r="B13" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13" t="s">
+        <v>32</v>
+      </c>
+      <c r="D13" t="s">
         <v>33</v>
       </c>
-      <c r="C12" t="s">
-        <v>33</v>
-      </c>
-      <c r="D12" t="s">
+      <c r="E13" t="s">
         <v>34</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F13" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="86.4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A14">
+        <v>94</v>
+      </c>
+      <c r="B14" t="s">
         <v>35</v>
       </c>
-      <c r="F12" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="86.4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13">
-        <v>94</v>
-      </c>
-      <c r="B13" t="s">
+      <c r="C14" t="s">
+        <v>35</v>
+      </c>
+      <c r="D14" t="s">
         <v>36</v>
       </c>
-      <c r="C13" t="s">
-        <v>36</v>
-      </c>
-      <c r="D13" t="s">
-        <v>37</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F13" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A14">
-        <v>1</v>
-      </c>
-      <c r="B14" t="s">
-        <v>38</v>
-      </c>
-      <c r="C14" t="s">
-        <v>38</v>
-      </c>
-      <c r="D14" t="s">
-        <v>39</v>
-      </c>
-      <c r="E14" t="s">
-        <v>40</v>
+      <c r="E14" s="1" t="s">
+        <v>46</v>
       </c>
       <c r="F14" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -909,19 +918,19 @@
         <v>1</v>
       </c>
       <c r="B15" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C15" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="D15" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="E15" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F15" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -929,19 +938,39 @@
         <v>1</v>
       </c>
       <c r="B16" t="s">
+        <v>64</v>
+      </c>
+      <c r="C16" t="s">
+        <v>64</v>
+      </c>
+      <c r="D16" t="s">
+        <v>40</v>
+      </c>
+      <c r="E16" t="s">
+        <v>41</v>
+      </c>
+      <c r="F16" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A17">
+        <v>1</v>
+      </c>
+      <c r="B17" t="s">
+        <v>42</v>
+      </c>
+      <c r="C17" t="s">
+        <v>42</v>
+      </c>
+      <c r="D17" t="s">
+        <v>43</v>
+      </c>
+      <c r="E17" t="s">
         <v>44</v>
       </c>
-      <c r="C16" t="s">
-        <v>44</v>
-      </c>
-      <c r="D16" t="s">
-        <v>45</v>
-      </c>
-      <c r="E16" t="s">
-        <v>46</v>
-      </c>
-      <c r="F16" t="s">
-        <v>55</v>
+      <c r="F17" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Change pads to 0603 and move some resistors around. This commit marks final draft
</commit_message>
<xml_diff>
--- a/eagle/bom/bom_jlc.xlsx
+++ b/eagle/bom/bom_jlc.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wpi0-my.sharepoint.com/personal/jwbuchta_wpi_edu/Documents/Jobs/academic_technician/flashing_led/eagle/bom/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="55" documentId="11_F25DC773A252ABDACC10483079DB61465BDE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3F7FC781-0DD2-47B6-A75D-F3371DF1DBAB}"/>
+  <xr:revisionPtr revIDLastSave="76" documentId="11_F25DC773A252ABDACC10483079DB61465BDE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4F3AF258-C576-4A66-98F7-857D3E64E2BF}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="68">
   <si>
     <t>Qty</t>
   </si>
@@ -60,12 +60,6 @@
   </si>
   <si>
     <t>Q1, Q2, Q3, Q4, Q5, Q6, QB, QG, QR</t>
-  </si>
-  <si>
-    <t>R-US_R0402</t>
-  </si>
-  <si>
-    <t>R0402</t>
   </si>
   <si>
     <t>100</t>
@@ -221,30 +215,12 @@
     <t>C2150</t>
   </si>
   <si>
-    <t>C25900</t>
-  </si>
-  <si>
-    <t>C25076</t>
-  </si>
-  <si>
-    <t>C25570</t>
-  </si>
-  <si>
-    <t>C25117</t>
-  </si>
-  <si>
-    <t>C24966</t>
-  </si>
-  <si>
     <t>TPS63000DRCR</t>
   </si>
   <si>
     <t>680k</t>
   </si>
   <si>
-    <t>C4131</t>
-  </si>
-  <si>
     <t>R76</t>
   </si>
   <si>
@@ -252,16 +228,43 @@
   </si>
   <si>
     <t>C2, C4, C7, C8</t>
+  </si>
+  <si>
+    <t>R0603</t>
+  </si>
+  <si>
+    <t>C23179</t>
+  </si>
+  <si>
+    <t>C25822</t>
+  </si>
+  <si>
+    <t>R-US_R0603</t>
+  </si>
+  <si>
+    <t>C23242</t>
+  </si>
+  <si>
+    <t>C23162</t>
+  </si>
+  <si>
+    <t>C2876573</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -638,7 +641,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -650,7 +653,7 @@
         <v>3</v>
       </c>
       <c r="F1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -670,7 +673,7 @@
         <v>7</v>
       </c>
       <c r="F2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="72" x14ac:dyDescent="0.55000000000000004">
@@ -681,16 +684,16 @@
         <v>470</v>
       </c>
       <c r="C3" t="s">
-        <v>8</v>
+        <v>64</v>
       </c>
       <c r="D3" t="s">
-        <v>9</v>
+        <v>61</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -698,19 +701,19 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>8</v>
+        <v>64</v>
       </c>
       <c r="D4" t="s">
+        <v>61</v>
+      </c>
+      <c r="E4" t="s">
         <v>9</v>
       </c>
-      <c r="E4" t="s">
-        <v>11</v>
-      </c>
       <c r="F4" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -718,19 +721,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" t="s">
         <v>12</v>
       </c>
-      <c r="C5" t="s">
+      <c r="E5" t="s">
         <v>13</v>
       </c>
-      <c r="D5" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" t="s">
-        <v>15</v>
-      </c>
       <c r="F5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -738,19 +741,19 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" t="s">
         <v>16</v>
       </c>
-      <c r="C6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" t="s">
-        <v>18</v>
-      </c>
       <c r="E6" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="F6" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -758,19 +761,19 @@
         <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>8</v>
+        <v>64</v>
       </c>
       <c r="D7" t="s">
-        <v>9</v>
+        <v>61</v>
       </c>
       <c r="E7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F7" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -778,19 +781,19 @@
         <v>1</v>
       </c>
       <c r="B8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" t="s">
         <v>21</v>
       </c>
-      <c r="C8" t="s">
-        <v>21</v>
-      </c>
-      <c r="D8" t="s">
-        <v>22</v>
-      </c>
-      <c r="E8" t="s">
-        <v>23</v>
-      </c>
       <c r="F8" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -798,19 +801,19 @@
         <v>1</v>
       </c>
       <c r="B9" t="s">
+        <v>57</v>
+      </c>
+      <c r="C9" t="s">
         <v>64</v>
       </c>
-      <c r="C9" t="s">
-        <v>8</v>
-      </c>
       <c r="D9" t="s">
-        <v>9</v>
+        <v>61</v>
       </c>
       <c r="E9" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="F9" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -818,19 +821,19 @@
         <v>4</v>
       </c>
       <c r="B10" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C10" t="s">
-        <v>8</v>
+        <v>64</v>
       </c>
       <c r="D10" t="s">
-        <v>9</v>
+        <v>61</v>
       </c>
       <c r="E10" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="F10" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -838,19 +841,19 @@
         <v>1</v>
       </c>
       <c r="B11" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" t="s">
         <v>25</v>
       </c>
-      <c r="C11" t="s">
-        <v>25</v>
-      </c>
-      <c r="D11" t="s">
-        <v>26</v>
-      </c>
-      <c r="E11" t="s">
-        <v>27</v>
-      </c>
       <c r="F11" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -858,19 +861,19 @@
         <v>1</v>
       </c>
       <c r="B12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" t="s">
         <v>28</v>
       </c>
-      <c r="C12" t="s">
-        <v>28</v>
-      </c>
-      <c r="D12" t="s">
-        <v>29</v>
-      </c>
-      <c r="E12" t="s">
-        <v>30</v>
-      </c>
       <c r="F12" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -878,19 +881,19 @@
         <v>1</v>
       </c>
       <c r="B13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13" t="s">
+        <v>30</v>
+      </c>
+      <c r="E13" t="s">
         <v>31</v>
       </c>
-      <c r="C13" t="s">
-        <v>31</v>
-      </c>
-      <c r="D13" t="s">
-        <v>32</v>
-      </c>
-      <c r="E13" t="s">
-        <v>33</v>
-      </c>
       <c r="F13" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="86.4" x14ac:dyDescent="0.55000000000000004">
@@ -898,19 +901,19 @@
         <v>94</v>
       </c>
       <c r="B14" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C14" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F14" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -918,19 +921,19 @@
         <v>1</v>
       </c>
       <c r="B15" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15" t="s">
+        <v>34</v>
+      </c>
+      <c r="D15" t="s">
+        <v>35</v>
+      </c>
+      <c r="E15" t="s">
         <v>36</v>
       </c>
-      <c r="C15" t="s">
-        <v>36</v>
-      </c>
-      <c r="D15" t="s">
-        <v>37</v>
-      </c>
-      <c r="E15" t="s">
-        <v>38</v>
-      </c>
       <c r="F15" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -938,19 +941,19 @@
         <v>1</v>
       </c>
       <c r="B16" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="C16" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="D16" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E16" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F16" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -958,22 +961,23 @@
         <v>1</v>
       </c>
       <c r="B17" t="s">
+        <v>39</v>
+      </c>
+      <c r="C17" t="s">
+        <v>39</v>
+      </c>
+      <c r="D17" t="s">
+        <v>40</v>
+      </c>
+      <c r="E17" t="s">
         <v>41</v>
       </c>
-      <c r="C17" t="s">
-        <v>41</v>
-      </c>
-      <c r="D17" t="s">
-        <v>42</v>
-      </c>
-      <c r="E17" t="s">
-        <v>43</v>
-      </c>
       <c r="F17" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">

</xml_diff>